<commit_message>
Final version of the projrct followup
</commit_message>
<xml_diff>
--- a/Suivi de projet.xlsx
+++ b/Suivi de projet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Personel\SpaceShooter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{723A579A-6A47-4A89-B32D-4817E6F6CE12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A60D501-0937-40C2-A5C3-B7797EF21D5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2D8ED4CF-38A5-4CA5-A364-F08410BB3B1F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="68">
   <si>
     <t>Taches</t>
   </si>
@@ -240,6 +240,9 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t>13/10/2026</t>
   </si>
 </sst>
 </file>
@@ -281,7 +284,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -501,11 +504,24 @@
         <color indexed="64"/>
       </diagonal>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -531,6 +547,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -540,11 +559,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -879,7 +912,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29FDCBCA-BB2D-43F7-9B5F-4B4D9B295C8E}">
-  <dimension ref="A1:AW57"/>
+  <dimension ref="A1:BM57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.42578125" style="1" customWidth="1"/>
@@ -907,84 +940,116 @@
     <col min="45" max="45" width="5.5703125" style="4" customWidth="1"/>
     <col min="46" max="48" width="5.5703125" customWidth="1"/>
     <col min="49" max="49" width="5.5703125" style="4" customWidth="1"/>
+    <col min="50" max="52" width="5.5703125" customWidth="1"/>
+    <col min="53" max="53" width="5.5703125" style="4" customWidth="1"/>
+    <col min="54" max="56" width="5.5703125" customWidth="1"/>
+    <col min="57" max="57" width="5.5703125" style="4" customWidth="1"/>
+    <col min="58" max="60" width="5.5703125" customWidth="1"/>
+    <col min="61" max="61" width="5.5703125" style="4" customWidth="1"/>
+    <col min="62" max="64" width="5.5703125" customWidth="1"/>
+    <col min="65" max="65" width="5.5703125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" s="3" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:65" s="3" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="21" t="s">
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="21" t="s">
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="19">
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="20">
         <v>46031</v>
       </c>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="19" t="s">
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
+      <c r="Q1" s="21"/>
+      <c r="R1" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="S1" s="20"/>
-      <c r="T1" s="20"/>
-      <c r="U1" s="20"/>
-      <c r="V1" s="19">
+      <c r="S1" s="21"/>
+      <c r="T1" s="21"/>
+      <c r="U1" s="21"/>
+      <c r="V1" s="20">
         <v>46243</v>
       </c>
-      <c r="W1" s="20"/>
-      <c r="X1" s="20"/>
-      <c r="Y1" s="20"/>
-      <c r="Z1" s="19" t="s">
+      <c r="W1" s="21"/>
+      <c r="X1" s="21"/>
+      <c r="Y1" s="21"/>
+      <c r="Z1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="AA1" s="20"/>
-      <c r="AB1" s="20"/>
-      <c r="AC1" s="20"/>
-      <c r="AD1" s="19" t="s">
+      <c r="AA1" s="21"/>
+      <c r="AB1" s="21"/>
+      <c r="AC1" s="21"/>
+      <c r="AD1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="AE1" s="20"/>
-      <c r="AF1" s="20"/>
-      <c r="AG1" s="20"/>
-      <c r="AH1" s="19" t="s">
+      <c r="AE1" s="21"/>
+      <c r="AF1" s="21"/>
+      <c r="AG1" s="21"/>
+      <c r="AH1" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="AI1" s="20"/>
-      <c r="AJ1" s="20"/>
-      <c r="AK1" s="20"/>
-      <c r="AL1" s="19" t="s">
+      <c r="AI1" s="21"/>
+      <c r="AJ1" s="21"/>
+      <c r="AK1" s="21"/>
+      <c r="AL1" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="AM1" s="20"/>
-      <c r="AN1" s="20"/>
-      <c r="AO1" s="20"/>
-      <c r="AP1" s="19" t="s">
+      <c r="AM1" s="21"/>
+      <c r="AN1" s="21"/>
+      <c r="AO1" s="21"/>
+      <c r="AP1" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="AQ1" s="20"/>
-      <c r="AR1" s="20"/>
-      <c r="AS1" s="20"/>
-      <c r="AT1" s="19" t="s">
+      <c r="AQ1" s="21"/>
+      <c r="AR1" s="21"/>
+      <c r="AS1" s="21"/>
+      <c r="AT1" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="AU1" s="20"/>
-      <c r="AV1" s="20"/>
-      <c r="AW1" s="20"/>
-    </row>
-    <row r="2" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AU1" s="23"/>
+      <c r="AV1" s="23"/>
+      <c r="AW1" s="24"/>
+      <c r="AX1" s="20">
+        <v>46152</v>
+      </c>
+      <c r="AY1" s="23"/>
+      <c r="AZ1" s="23"/>
+      <c r="BA1" s="23"/>
+      <c r="BB1" s="20">
+        <v>46183</v>
+      </c>
+      <c r="BC1" s="23"/>
+      <c r="BD1" s="23"/>
+      <c r="BE1" s="23"/>
+      <c r="BF1" s="20">
+        <v>46366</v>
+      </c>
+      <c r="BG1" s="23"/>
+      <c r="BH1" s="23"/>
+      <c r="BI1" s="23"/>
+      <c r="BJ1" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="BK1" s="23"/>
+      <c r="BL1" s="23"/>
+      <c r="BM1" s="23"/>
+    </row>
+    <row r="2" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
@@ -1036,8 +1101,24 @@
       <c r="AU2" s="7"/>
       <c r="AV2" s="7"/>
       <c r="AW2" s="8"/>
-    </row>
-    <row r="3" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX2" s="7"/>
+      <c r="AY2" s="7"/>
+      <c r="AZ2" s="7"/>
+      <c r="BA2" s="8"/>
+      <c r="BB2" s="7"/>
+      <c r="BC2" s="7"/>
+      <c r="BD2" s="7"/>
+      <c r="BE2" s="8"/>
+      <c r="BF2" s="7"/>
+      <c r="BG2" s="7"/>
+      <c r="BH2" s="7"/>
+      <c r="BI2" s="8"/>
+      <c r="BJ2" s="7"/>
+      <c r="BK2" s="7"/>
+      <c r="BL2" s="7"/>
+      <c r="BM2" s="8"/>
+    </row>
+    <row r="3" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>59</v>
       </c>
@@ -1093,8 +1174,24 @@
       <c r="AU3" s="9"/>
       <c r="AV3" s="9"/>
       <c r="AW3" s="10"/>
-    </row>
-    <row r="4" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX3" s="11"/>
+      <c r="AY3" s="9"/>
+      <c r="AZ3" s="9"/>
+      <c r="BA3" s="10"/>
+      <c r="BB3" s="11"/>
+      <c r="BC3" s="9"/>
+      <c r="BD3" s="9"/>
+      <c r="BE3" s="10"/>
+      <c r="BF3" s="11"/>
+      <c r="BG3" s="9"/>
+      <c r="BH3" s="9"/>
+      <c r="BI3" s="10"/>
+      <c r="BJ3" s="11"/>
+      <c r="BK3" s="9"/>
+      <c r="BL3" s="9"/>
+      <c r="BM3" s="10"/>
+    </row>
+    <row r="4" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>60</v>
       </c>
@@ -1150,8 +1247,24 @@
       <c r="AU4" s="9"/>
       <c r="AV4" s="9"/>
       <c r="AW4" s="10"/>
-    </row>
-    <row r="5" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX4" s="11"/>
+      <c r="AY4" s="9"/>
+      <c r="AZ4" s="9"/>
+      <c r="BA4" s="10"/>
+      <c r="BB4" s="11"/>
+      <c r="BC4" s="9"/>
+      <c r="BD4" s="9"/>
+      <c r="BE4" s="10"/>
+      <c r="BF4" s="11"/>
+      <c r="BG4" s="9"/>
+      <c r="BH4" s="9"/>
+      <c r="BI4" s="10"/>
+      <c r="BJ4" s="11"/>
+      <c r="BK4" s="9"/>
+      <c r="BL4" s="9"/>
+      <c r="BM4" s="10"/>
+    </row>
+    <row r="5" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>61</v>
       </c>
@@ -1205,8 +1318,24 @@
       <c r="AU5" s="9"/>
       <c r="AV5" s="9"/>
       <c r="AW5" s="10"/>
-    </row>
-    <row r="6" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX5" s="11"/>
+      <c r="AY5" s="9"/>
+      <c r="AZ5" s="9"/>
+      <c r="BA5" s="10"/>
+      <c r="BB5" s="11"/>
+      <c r="BC5" s="9"/>
+      <c r="BD5" s="9"/>
+      <c r="BE5" s="10"/>
+      <c r="BF5" s="11"/>
+      <c r="BG5" s="9"/>
+      <c r="BH5" s="9"/>
+      <c r="BI5" s="10"/>
+      <c r="BJ5" s="11"/>
+      <c r="BK5" s="9"/>
+      <c r="BL5" s="9"/>
+      <c r="BM5" s="10"/>
+    </row>
+    <row r="6" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
@@ -1262,8 +1391,24 @@
       <c r="AU6" s="9"/>
       <c r="AV6" s="9"/>
       <c r="AW6" s="10"/>
-    </row>
-    <row r="7" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX6" s="11"/>
+      <c r="AY6" s="9"/>
+      <c r="AZ6" s="9"/>
+      <c r="BA6" s="10"/>
+      <c r="BB6" s="11"/>
+      <c r="BC6" s="9"/>
+      <c r="BD6" s="9"/>
+      <c r="BE6" s="10"/>
+      <c r="BF6" s="11"/>
+      <c r="BG6" s="9"/>
+      <c r="BH6" s="9"/>
+      <c r="BI6" s="10"/>
+      <c r="BJ6" s="11"/>
+      <c r="BK6" s="9"/>
+      <c r="BL6" s="9"/>
+      <c r="BM6" s="10"/>
+    </row>
+    <row r="7" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -1315,8 +1460,24 @@
       <c r="AU7" s="9"/>
       <c r="AV7" s="9"/>
       <c r="AW7" s="10"/>
-    </row>
-    <row r="8" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX7" s="11"/>
+      <c r="AY7" s="9"/>
+      <c r="AZ7" s="9"/>
+      <c r="BA7" s="10"/>
+      <c r="BB7" s="11"/>
+      <c r="BC7" s="9"/>
+      <c r="BD7" s="9"/>
+      <c r="BE7" s="10"/>
+      <c r="BF7" s="11"/>
+      <c r="BG7" s="9"/>
+      <c r="BH7" s="9"/>
+      <c r="BI7" s="10"/>
+      <c r="BJ7" s="11"/>
+      <c r="BK7" s="9"/>
+      <c r="BL7" s="9"/>
+      <c r="BM7" s="10"/>
+    </row>
+    <row r="8" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
@@ -1368,8 +1529,24 @@
       <c r="AU8" s="9"/>
       <c r="AV8" s="9"/>
       <c r="AW8" s="10"/>
-    </row>
-    <row r="9" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX8" s="11"/>
+      <c r="AY8" s="9"/>
+      <c r="AZ8" s="9"/>
+      <c r="BA8" s="10"/>
+      <c r="BB8" s="11"/>
+      <c r="BC8" s="9"/>
+      <c r="BD8" s="9"/>
+      <c r="BE8" s="10"/>
+      <c r="BF8" s="11"/>
+      <c r="BG8" s="9"/>
+      <c r="BH8" s="9"/>
+      <c r="BI8" s="10"/>
+      <c r="BJ8" s="11"/>
+      <c r="BK8" s="9"/>
+      <c r="BL8" s="9"/>
+      <c r="BM8" s="10"/>
+    </row>
+    <row r="9" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
@@ -1427,8 +1604,24 @@
       <c r="AU9" s="9"/>
       <c r="AV9" s="9"/>
       <c r="AW9" s="10"/>
-    </row>
-    <row r="10" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX9" s="11"/>
+      <c r="AY9" s="9"/>
+      <c r="AZ9" s="9"/>
+      <c r="BA9" s="10"/>
+      <c r="BB9" s="11"/>
+      <c r="BC9" s="9"/>
+      <c r="BD9" s="9"/>
+      <c r="BE9" s="10"/>
+      <c r="BF9" s="11"/>
+      <c r="BG9" s="9"/>
+      <c r="BH9" s="9"/>
+      <c r="BI9" s="10"/>
+      <c r="BJ9" s="11"/>
+      <c r="BK9" s="9"/>
+      <c r="BL9" s="9"/>
+      <c r="BM9" s="10"/>
+    </row>
+    <row r="10" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
@@ -1488,8 +1681,24 @@
       <c r="AU10" s="9"/>
       <c r="AV10" s="9"/>
       <c r="AW10" s="10"/>
-    </row>
-    <row r="11" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX10" s="11"/>
+      <c r="AY10" s="9"/>
+      <c r="AZ10" s="9"/>
+      <c r="BA10" s="10"/>
+      <c r="BB10" s="11"/>
+      <c r="BC10" s="9"/>
+      <c r="BD10" s="9"/>
+      <c r="BE10" s="10"/>
+      <c r="BF10" s="11"/>
+      <c r="BG10" s="9"/>
+      <c r="BH10" s="9"/>
+      <c r="BI10" s="10"/>
+      <c r="BJ10" s="11"/>
+      <c r="BK10" s="9"/>
+      <c r="BL10" s="9"/>
+      <c r="BM10" s="10"/>
+    </row>
+    <row r="11" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>14</v>
       </c>
@@ -1543,8 +1752,24 @@
       <c r="AU11" s="9"/>
       <c r="AV11" s="9"/>
       <c r="AW11" s="10"/>
-    </row>
-    <row r="12" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX11" s="11"/>
+      <c r="AY11" s="9"/>
+      <c r="AZ11" s="9"/>
+      <c r="BA11" s="10"/>
+      <c r="BB11" s="11"/>
+      <c r="BC11" s="9"/>
+      <c r="BD11" s="9"/>
+      <c r="BE11" s="10"/>
+      <c r="BF11" s="11"/>
+      <c r="BG11" s="9"/>
+      <c r="BH11" s="9"/>
+      <c r="BI11" s="10"/>
+      <c r="BJ11" s="11"/>
+      <c r="BK11" s="9"/>
+      <c r="BL11" s="9"/>
+      <c r="BM11" s="10"/>
+    </row>
+    <row r="12" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>15</v>
       </c>
@@ -1598,8 +1823,24 @@
       <c r="AU12" s="9"/>
       <c r="AV12" s="9"/>
       <c r="AW12" s="10"/>
-    </row>
-    <row r="13" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX12" s="11"/>
+      <c r="AY12" s="9"/>
+      <c r="AZ12" s="9"/>
+      <c r="BA12" s="10"/>
+      <c r="BB12" s="11"/>
+      <c r="BC12" s="9"/>
+      <c r="BD12" s="9"/>
+      <c r="BE12" s="10"/>
+      <c r="BF12" s="11"/>
+      <c r="BG12" s="9"/>
+      <c r="BH12" s="9"/>
+      <c r="BI12" s="10"/>
+      <c r="BJ12" s="11"/>
+      <c r="BK12" s="9"/>
+      <c r="BL12" s="9"/>
+      <c r="BM12" s="10"/>
+    </row>
+    <row r="13" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
@@ -1653,8 +1894,24 @@
       <c r="AU13" s="9"/>
       <c r="AV13" s="9"/>
       <c r="AW13" s="10"/>
-    </row>
-    <row r="14" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX13" s="11"/>
+      <c r="AY13" s="9"/>
+      <c r="AZ13" s="9"/>
+      <c r="BA13" s="10"/>
+      <c r="BB13" s="11"/>
+      <c r="BC13" s="9"/>
+      <c r="BD13" s="9"/>
+      <c r="BE13" s="10"/>
+      <c r="BF13" s="11"/>
+      <c r="BG13" s="9"/>
+      <c r="BH13" s="9"/>
+      <c r="BI13" s="10"/>
+      <c r="BJ13" s="11"/>
+      <c r="BK13" s="9"/>
+      <c r="BL13" s="9"/>
+      <c r="BM13" s="10"/>
+    </row>
+    <row r="14" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>17</v>
       </c>
@@ -1708,8 +1965,24 @@
       <c r="AU14" s="9"/>
       <c r="AV14" s="9"/>
       <c r="AW14" s="10"/>
-    </row>
-    <row r="15" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX14" s="11"/>
+      <c r="AY14" s="9"/>
+      <c r="AZ14" s="9"/>
+      <c r="BA14" s="10"/>
+      <c r="BB14" s="11"/>
+      <c r="BC14" s="9"/>
+      <c r="BD14" s="9"/>
+      <c r="BE14" s="10"/>
+      <c r="BF14" s="11"/>
+      <c r="BG14" s="9"/>
+      <c r="BH14" s="9"/>
+      <c r="BI14" s="10"/>
+      <c r="BJ14" s="11"/>
+      <c r="BK14" s="9"/>
+      <c r="BL14" s="9"/>
+      <c r="BM14" s="10"/>
+    </row>
+    <row r="15" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>18</v>
       </c>
@@ -1765,8 +2038,24 @@
       <c r="AU15" s="9"/>
       <c r="AV15" s="9"/>
       <c r="AW15" s="10"/>
-    </row>
-    <row r="16" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX15" s="11"/>
+      <c r="AY15" s="9"/>
+      <c r="AZ15" s="9"/>
+      <c r="BA15" s="10"/>
+      <c r="BB15" s="11"/>
+      <c r="BC15" s="9"/>
+      <c r="BD15" s="9"/>
+      <c r="BE15" s="10"/>
+      <c r="BF15" s="11"/>
+      <c r="BG15" s="9"/>
+      <c r="BH15" s="9"/>
+      <c r="BI15" s="10"/>
+      <c r="BJ15" s="11"/>
+      <c r="BK15" s="9"/>
+      <c r="BL15" s="9"/>
+      <c r="BM15" s="10"/>
+    </row>
+    <row r="16" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
@@ -1820,8 +2109,24 @@
       <c r="AU16" s="9"/>
       <c r="AV16" s="9"/>
       <c r="AW16" s="10"/>
-    </row>
-    <row r="17" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX16" s="11"/>
+      <c r="AY16" s="9"/>
+      <c r="AZ16" s="9"/>
+      <c r="BA16" s="10"/>
+      <c r="BB16" s="11"/>
+      <c r="BC16" s="9"/>
+      <c r="BD16" s="9"/>
+      <c r="BE16" s="10"/>
+      <c r="BF16" s="11"/>
+      <c r="BG16" s="9"/>
+      <c r="BH16" s="9"/>
+      <c r="BI16" s="10"/>
+      <c r="BJ16" s="11"/>
+      <c r="BK16" s="9"/>
+      <c r="BL16" s="9"/>
+      <c r="BM16" s="10"/>
+    </row>
+    <row r="17" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
@@ -1877,8 +2182,24 @@
       <c r="AU17" s="9"/>
       <c r="AV17" s="9"/>
       <c r="AW17" s="10"/>
-    </row>
-    <row r="18" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX17" s="11"/>
+      <c r="AY17" s="9"/>
+      <c r="AZ17" s="9"/>
+      <c r="BA17" s="10"/>
+      <c r="BB17" s="11"/>
+      <c r="BC17" s="9"/>
+      <c r="BD17" s="9"/>
+      <c r="BE17" s="10"/>
+      <c r="BF17" s="11"/>
+      <c r="BG17" s="9"/>
+      <c r="BH17" s="9"/>
+      <c r="BI17" s="10"/>
+      <c r="BJ17" s="11"/>
+      <c r="BK17" s="9"/>
+      <c r="BL17" s="9"/>
+      <c r="BM17" s="10"/>
+    </row>
+    <row r="18" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>21</v>
       </c>
@@ -1934,8 +2255,24 @@
       <c r="AU18" s="9"/>
       <c r="AV18" s="9"/>
       <c r="AW18" s="10"/>
-    </row>
-    <row r="19" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX18" s="11"/>
+      <c r="AY18" s="9"/>
+      <c r="AZ18" s="9"/>
+      <c r="BA18" s="10"/>
+      <c r="BB18" s="11"/>
+      <c r="BC18" s="9"/>
+      <c r="BD18" s="9"/>
+      <c r="BE18" s="10"/>
+      <c r="BF18" s="11"/>
+      <c r="BG18" s="9"/>
+      <c r="BH18" s="9"/>
+      <c r="BI18" s="10"/>
+      <c r="BJ18" s="11"/>
+      <c r="BK18" s="9"/>
+      <c r="BL18" s="9"/>
+      <c r="BM18" s="10"/>
+    </row>
+    <row r="19" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>22</v>
       </c>
@@ -1989,8 +2326,24 @@
       <c r="AU19" s="9"/>
       <c r="AV19" s="9"/>
       <c r="AW19" s="10"/>
-    </row>
-    <row r="20" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX19" s="11"/>
+      <c r="AY19" s="9"/>
+      <c r="AZ19" s="9"/>
+      <c r="BA19" s="10"/>
+      <c r="BB19" s="11"/>
+      <c r="BC19" s="9"/>
+      <c r="BD19" s="9"/>
+      <c r="BE19" s="10"/>
+      <c r="BF19" s="11"/>
+      <c r="BG19" s="9"/>
+      <c r="BH19" s="9"/>
+      <c r="BI19" s="10"/>
+      <c r="BJ19" s="11"/>
+      <c r="BK19" s="9"/>
+      <c r="BL19" s="9"/>
+      <c r="BM19" s="10"/>
+    </row>
+    <row r="20" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>23</v>
       </c>
@@ -2044,8 +2397,24 @@
       <c r="AU20" s="9"/>
       <c r="AV20" s="9"/>
       <c r="AW20" s="10"/>
-    </row>
-    <row r="21" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX20" s="11"/>
+      <c r="AY20" s="9"/>
+      <c r="AZ20" s="9"/>
+      <c r="BA20" s="10"/>
+      <c r="BB20" s="11"/>
+      <c r="BC20" s="9"/>
+      <c r="BD20" s="9"/>
+      <c r="BE20" s="10"/>
+      <c r="BF20" s="11"/>
+      <c r="BG20" s="9"/>
+      <c r="BH20" s="9"/>
+      <c r="BI20" s="10"/>
+      <c r="BJ20" s="11"/>
+      <c r="BK20" s="9"/>
+      <c r="BL20" s="9"/>
+      <c r="BM20" s="10"/>
+    </row>
+    <row r="21" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>24</v>
       </c>
@@ -2101,8 +2470,24 @@
       <c r="AU21" s="9"/>
       <c r="AV21" s="9"/>
       <c r="AW21" s="10"/>
-    </row>
-    <row r="22" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX21" s="11"/>
+      <c r="AY21" s="9"/>
+      <c r="AZ21" s="9"/>
+      <c r="BA21" s="10"/>
+      <c r="BB21" s="11"/>
+      <c r="BC21" s="9"/>
+      <c r="BD21" s="9"/>
+      <c r="BE21" s="10"/>
+      <c r="BF21" s="11"/>
+      <c r="BG21" s="9"/>
+      <c r="BH21" s="9"/>
+      <c r="BI21" s="10"/>
+      <c r="BJ21" s="11"/>
+      <c r="BK21" s="9"/>
+      <c r="BL21" s="9"/>
+      <c r="BM21" s="10"/>
+    </row>
+    <row r="22" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>25</v>
       </c>
@@ -2158,8 +2543,24 @@
       <c r="AU22" s="9"/>
       <c r="AV22" s="9"/>
       <c r="AW22" s="10"/>
-    </row>
-    <row r="23" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX22" s="11"/>
+      <c r="AY22" s="9"/>
+      <c r="AZ22" s="9"/>
+      <c r="BA22" s="10"/>
+      <c r="BB22" s="11"/>
+      <c r="BC22" s="9"/>
+      <c r="BD22" s="9"/>
+      <c r="BE22" s="10"/>
+      <c r="BF22" s="11"/>
+      <c r="BG22" s="9"/>
+      <c r="BH22" s="9"/>
+      <c r="BI22" s="10"/>
+      <c r="BJ22" s="11"/>
+      <c r="BK22" s="9"/>
+      <c r="BL22" s="9"/>
+      <c r="BM22" s="10"/>
+    </row>
+    <row r="23" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>26</v>
       </c>
@@ -2215,8 +2616,24 @@
       <c r="AU23" s="9"/>
       <c r="AV23" s="9"/>
       <c r="AW23" s="10"/>
-    </row>
-    <row r="24" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX23" s="11"/>
+      <c r="AY23" s="9"/>
+      <c r="AZ23" s="9"/>
+      <c r="BA23" s="10"/>
+      <c r="BB23" s="11"/>
+      <c r="BC23" s="9"/>
+      <c r="BD23" s="9"/>
+      <c r="BE23" s="10"/>
+      <c r="BF23" s="11"/>
+      <c r="BG23" s="9"/>
+      <c r="BH23" s="9"/>
+      <c r="BI23" s="10"/>
+      <c r="BJ23" s="11"/>
+      <c r="BK23" s="9"/>
+      <c r="BL23" s="9"/>
+      <c r="BM23" s="10"/>
+    </row>
+    <row r="24" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>27</v>
       </c>
@@ -2272,8 +2689,24 @@
       <c r="AU24" s="9"/>
       <c r="AV24" s="9"/>
       <c r="AW24" s="10"/>
-    </row>
-    <row r="25" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX24" s="11"/>
+      <c r="AY24" s="9"/>
+      <c r="AZ24" s="9"/>
+      <c r="BA24" s="10"/>
+      <c r="BB24" s="11"/>
+      <c r="BC24" s="9"/>
+      <c r="BD24" s="9"/>
+      <c r="BE24" s="10"/>
+      <c r="BF24" s="11"/>
+      <c r="BG24" s="9"/>
+      <c r="BH24" s="9"/>
+      <c r="BI24" s="10"/>
+      <c r="BJ24" s="11"/>
+      <c r="BK24" s="9"/>
+      <c r="BL24" s="9"/>
+      <c r="BM24" s="10"/>
+    </row>
+    <row r="25" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>28</v>
       </c>
@@ -2329,8 +2762,24 @@
       <c r="AU25" s="9"/>
       <c r="AV25" s="9"/>
       <c r="AW25" s="10"/>
-    </row>
-    <row r="26" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX25" s="11"/>
+      <c r="AY25" s="9"/>
+      <c r="AZ25" s="9"/>
+      <c r="BA25" s="10"/>
+      <c r="BB25" s="11"/>
+      <c r="BC25" s="9"/>
+      <c r="BD25" s="9"/>
+      <c r="BE25" s="10"/>
+      <c r="BF25" s="11"/>
+      <c r="BG25" s="9"/>
+      <c r="BH25" s="9"/>
+      <c r="BI25" s="10"/>
+      <c r="BJ25" s="11"/>
+      <c r="BK25" s="9"/>
+      <c r="BL25" s="9"/>
+      <c r="BM25" s="10"/>
+    </row>
+    <row r="26" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>29</v>
       </c>
@@ -2386,8 +2835,24 @@
       <c r="AU26" s="9"/>
       <c r="AV26" s="9"/>
       <c r="AW26" s="10"/>
-    </row>
-    <row r="27" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX26" s="11"/>
+      <c r="AY26" s="9"/>
+      <c r="AZ26" s="9"/>
+      <c r="BA26" s="10"/>
+      <c r="BB26" s="11"/>
+      <c r="BC26" s="9"/>
+      <c r="BD26" s="9"/>
+      <c r="BE26" s="10"/>
+      <c r="BF26" s="11"/>
+      <c r="BG26" s="9"/>
+      <c r="BH26" s="9"/>
+      <c r="BI26" s="10"/>
+      <c r="BJ26" s="11"/>
+      <c r="BK26" s="9"/>
+      <c r="BL26" s="9"/>
+      <c r="BM26" s="10"/>
+    </row>
+    <row r="27" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>30</v>
       </c>
@@ -2441,8 +2906,24 @@
       <c r="AU27" s="9"/>
       <c r="AV27" s="9"/>
       <c r="AW27" s="10"/>
-    </row>
-    <row r="28" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX27" s="11"/>
+      <c r="AY27" s="9"/>
+      <c r="AZ27" s="9"/>
+      <c r="BA27" s="10"/>
+      <c r="BB27" s="11"/>
+      <c r="BC27" s="9"/>
+      <c r="BD27" s="9"/>
+      <c r="BE27" s="10"/>
+      <c r="BF27" s="11"/>
+      <c r="BG27" s="9"/>
+      <c r="BH27" s="9"/>
+      <c r="BI27" s="10"/>
+      <c r="BJ27" s="11"/>
+      <c r="BK27" s="9"/>
+      <c r="BL27" s="9"/>
+      <c r="BM27" s="10"/>
+    </row>
+    <row r="28" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>31</v>
       </c>
@@ -2498,8 +2979,24 @@
       <c r="AU28" s="9"/>
       <c r="AV28" s="9"/>
       <c r="AW28" s="10"/>
-    </row>
-    <row r="29" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX28" s="11"/>
+      <c r="AY28" s="9"/>
+      <c r="AZ28" s="9"/>
+      <c r="BA28" s="10"/>
+      <c r="BB28" s="11"/>
+      <c r="BC28" s="9"/>
+      <c r="BD28" s="9"/>
+      <c r="BE28" s="10"/>
+      <c r="BF28" s="11"/>
+      <c r="BG28" s="9"/>
+      <c r="BH28" s="9"/>
+      <c r="BI28" s="10"/>
+      <c r="BJ28" s="11"/>
+      <c r="BK28" s="9"/>
+      <c r="BL28" s="9"/>
+      <c r="BM28" s="10"/>
+    </row>
+    <row r="29" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>32</v>
       </c>
@@ -2555,8 +3052,24 @@
       <c r="AU29" s="9"/>
       <c r="AV29" s="9"/>
       <c r="AW29" s="10"/>
-    </row>
-    <row r="30" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX29" s="11"/>
+      <c r="AY29" s="9"/>
+      <c r="AZ29" s="9"/>
+      <c r="BA29" s="10"/>
+      <c r="BB29" s="11"/>
+      <c r="BC29" s="9"/>
+      <c r="BD29" s="9"/>
+      <c r="BE29" s="10"/>
+      <c r="BF29" s="11"/>
+      <c r="BG29" s="9"/>
+      <c r="BH29" s="9"/>
+      <c r="BI29" s="10"/>
+      <c r="BJ29" s="11"/>
+      <c r="BK29" s="9"/>
+      <c r="BL29" s="9"/>
+      <c r="BM29" s="10"/>
+    </row>
+    <row r="30" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>33</v>
       </c>
@@ -2608,8 +3121,24 @@
       <c r="AU30" s="9"/>
       <c r="AV30" s="9"/>
       <c r="AW30" s="10"/>
-    </row>
-    <row r="31" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX30" s="11"/>
+      <c r="AY30" s="9"/>
+      <c r="AZ30" s="9"/>
+      <c r="BA30" s="10"/>
+      <c r="BB30" s="11"/>
+      <c r="BC30" s="9"/>
+      <c r="BD30" s="9"/>
+      <c r="BE30" s="10"/>
+      <c r="BF30" s="11"/>
+      <c r="BG30" s="9"/>
+      <c r="BH30" s="9"/>
+      <c r="BI30" s="10"/>
+      <c r="BJ30" s="11"/>
+      <c r="BK30" s="9"/>
+      <c r="BL30" s="9"/>
+      <c r="BM30" s="10"/>
+    </row>
+    <row r="31" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>34</v>
       </c>
@@ -2661,8 +3190,24 @@
       <c r="AU31" s="9"/>
       <c r="AV31" s="9"/>
       <c r="AW31" s="10"/>
-    </row>
-    <row r="32" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX31" s="11"/>
+      <c r="AY31" s="9"/>
+      <c r="AZ31" s="9"/>
+      <c r="BA31" s="10"/>
+      <c r="BB31" s="11"/>
+      <c r="BC31" s="9"/>
+      <c r="BD31" s="9"/>
+      <c r="BE31" s="10"/>
+      <c r="BF31" s="11"/>
+      <c r="BG31" s="9"/>
+      <c r="BH31" s="9"/>
+      <c r="BI31" s="10"/>
+      <c r="BJ31" s="11"/>
+      <c r="BK31" s="9"/>
+      <c r="BL31" s="9"/>
+      <c r="BM31" s="10"/>
+    </row>
+    <row r="32" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>35</v>
       </c>
@@ -2718,8 +3263,24 @@
       <c r="AU32" s="9"/>
       <c r="AV32" s="9"/>
       <c r="AW32" s="10"/>
-    </row>
-    <row r="33" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX32" s="11"/>
+      <c r="AY32" s="9"/>
+      <c r="AZ32" s="9"/>
+      <c r="BA32" s="10"/>
+      <c r="BB32" s="11"/>
+      <c r="BC32" s="9"/>
+      <c r="BD32" s="9"/>
+      <c r="BE32" s="10"/>
+      <c r="BF32" s="11"/>
+      <c r="BG32" s="9"/>
+      <c r="BH32" s="9"/>
+      <c r="BI32" s="10"/>
+      <c r="BJ32" s="11"/>
+      <c r="BK32" s="9"/>
+      <c r="BL32" s="9"/>
+      <c r="BM32" s="10"/>
+    </row>
+    <row r="33" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>36</v>
       </c>
@@ -2771,8 +3332,24 @@
       <c r="AU33" s="9"/>
       <c r="AV33" s="9"/>
       <c r="AW33" s="10"/>
-    </row>
-    <row r="34" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX33" s="11"/>
+      <c r="AY33" s="9"/>
+      <c r="AZ33" s="9"/>
+      <c r="BA33" s="10"/>
+      <c r="BB33" s="11"/>
+      <c r="BC33" s="9"/>
+      <c r="BD33" s="9"/>
+      <c r="BE33" s="10"/>
+      <c r="BF33" s="11"/>
+      <c r="BG33" s="9"/>
+      <c r="BH33" s="9"/>
+      <c r="BI33" s="10"/>
+      <c r="BJ33" s="11"/>
+      <c r="BK33" s="9"/>
+      <c r="BL33" s="9"/>
+      <c r="BM33" s="10"/>
+    </row>
+    <row r="34" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>37</v>
       </c>
@@ -2824,8 +3401,24 @@
       <c r="AU34" s="9"/>
       <c r="AV34" s="9"/>
       <c r="AW34" s="10"/>
-    </row>
-    <row r="35" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX34" s="11"/>
+      <c r="AY34" s="9"/>
+      <c r="AZ34" s="9"/>
+      <c r="BA34" s="10"/>
+      <c r="BB34" s="11"/>
+      <c r="BC34" s="9"/>
+      <c r="BD34" s="9"/>
+      <c r="BE34" s="10"/>
+      <c r="BF34" s="11"/>
+      <c r="BG34" s="9"/>
+      <c r="BH34" s="9"/>
+      <c r="BI34" s="10"/>
+      <c r="BJ34" s="11"/>
+      <c r="BK34" s="9"/>
+      <c r="BL34" s="9"/>
+      <c r="BM34" s="10"/>
+    </row>
+    <row r="35" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>38</v>
       </c>
@@ -2877,8 +3470,24 @@
       <c r="AU35" s="9"/>
       <c r="AV35" s="9"/>
       <c r="AW35" s="10"/>
-    </row>
-    <row r="36" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX35" s="11"/>
+      <c r="AY35" s="9"/>
+      <c r="AZ35" s="9"/>
+      <c r="BA35" s="10"/>
+      <c r="BB35" s="11"/>
+      <c r="BC35" s="9"/>
+      <c r="BD35" s="9"/>
+      <c r="BE35" s="10"/>
+      <c r="BF35" s="11"/>
+      <c r="BG35" s="9"/>
+      <c r="BH35" s="9"/>
+      <c r="BI35" s="10"/>
+      <c r="BJ35" s="11"/>
+      <c r="BK35" s="9"/>
+      <c r="BL35" s="9"/>
+      <c r="BM35" s="10"/>
+    </row>
+    <row r="36" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>62</v>
       </c>
@@ -2934,8 +3543,24 @@
       <c r="AU36" s="9"/>
       <c r="AV36" s="9"/>
       <c r="AW36" s="10"/>
-    </row>
-    <row r="37" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX36" s="11"/>
+      <c r="AY36" s="9"/>
+      <c r="AZ36" s="9"/>
+      <c r="BA36" s="10"/>
+      <c r="BB36" s="11"/>
+      <c r="BC36" s="9"/>
+      <c r="BD36" s="9"/>
+      <c r="BE36" s="10"/>
+      <c r="BF36" s="11"/>
+      <c r="BG36" s="9"/>
+      <c r="BH36" s="9"/>
+      <c r="BI36" s="10"/>
+      <c r="BJ36" s="11"/>
+      <c r="BK36" s="9"/>
+      <c r="BL36" s="9"/>
+      <c r="BM36" s="10"/>
+    </row>
+    <row r="37" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>39</v>
       </c>
@@ -2989,8 +3614,24 @@
       <c r="AU37" s="9"/>
       <c r="AV37" s="9"/>
       <c r="AW37" s="10"/>
-    </row>
-    <row r="38" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX37" s="11"/>
+      <c r="AY37" s="9"/>
+      <c r="AZ37" s="9"/>
+      <c r="BA37" s="10"/>
+      <c r="BB37" s="11"/>
+      <c r="BC37" s="9"/>
+      <c r="BD37" s="9"/>
+      <c r="BE37" s="10"/>
+      <c r="BF37" s="11"/>
+      <c r="BG37" s="9"/>
+      <c r="BH37" s="9"/>
+      <c r="BI37" s="10"/>
+      <c r="BJ37" s="11"/>
+      <c r="BK37" s="9"/>
+      <c r="BL37" s="9"/>
+      <c r="BM37" s="10"/>
+    </row>
+    <row r="38" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>40</v>
       </c>
@@ -3050,8 +3691,24 @@
       <c r="AU38" s="9"/>
       <c r="AV38" s="9"/>
       <c r="AW38" s="10"/>
-    </row>
-    <row r="39" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX38" s="11"/>
+      <c r="AY38" s="9"/>
+      <c r="AZ38" s="9"/>
+      <c r="BA38" s="10"/>
+      <c r="BB38" s="11"/>
+      <c r="BC38" s="9"/>
+      <c r="BD38" s="9"/>
+      <c r="BE38" s="10"/>
+      <c r="BF38" s="11"/>
+      <c r="BG38" s="9"/>
+      <c r="BH38" s="9"/>
+      <c r="BI38" s="10"/>
+      <c r="BJ38" s="11"/>
+      <c r="BK38" s="9"/>
+      <c r="BL38" s="9"/>
+      <c r="BM38" s="10"/>
+    </row>
+    <row r="39" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>41</v>
       </c>
@@ -3105,8 +3762,24 @@
       <c r="AU39" s="9"/>
       <c r="AV39" s="9"/>
       <c r="AW39" s="10"/>
-    </row>
-    <row r="40" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX39" s="11"/>
+      <c r="AY39" s="9"/>
+      <c r="AZ39" s="9"/>
+      <c r="BA39" s="10"/>
+      <c r="BB39" s="11"/>
+      <c r="BC39" s="9"/>
+      <c r="BD39" s="9"/>
+      <c r="BE39" s="10"/>
+      <c r="BF39" s="11"/>
+      <c r="BG39" s="9"/>
+      <c r="BH39" s="9"/>
+      <c r="BI39" s="10"/>
+      <c r="BJ39" s="11"/>
+      <c r="BK39" s="9"/>
+      <c r="BL39" s="9"/>
+      <c r="BM39" s="10"/>
+    </row>
+    <row r="40" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>42</v>
       </c>
@@ -3162,8 +3835,24 @@
       <c r="AU40" s="9"/>
       <c r="AV40" s="9"/>
       <c r="AW40" s="10"/>
-    </row>
-    <row r="41" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX40" s="11"/>
+      <c r="AY40" s="9"/>
+      <c r="AZ40" s="9"/>
+      <c r="BA40" s="10"/>
+      <c r="BB40" s="11"/>
+      <c r="BC40" s="9"/>
+      <c r="BD40" s="9"/>
+      <c r="BE40" s="10"/>
+      <c r="BF40" s="11"/>
+      <c r="BG40" s="9"/>
+      <c r="BH40" s="9"/>
+      <c r="BI40" s="10"/>
+      <c r="BJ40" s="11"/>
+      <c r="BK40" s="9"/>
+      <c r="BL40" s="9"/>
+      <c r="BM40" s="10"/>
+    </row>
+    <row r="41" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>43</v>
       </c>
@@ -3215,8 +3904,24 @@
       <c r="AU41" s="13"/>
       <c r="AV41" s="13"/>
       <c r="AW41" s="15"/>
-    </row>
-    <row r="42" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX41" s="12"/>
+      <c r="AY41" s="13"/>
+      <c r="AZ41" s="13"/>
+      <c r="BA41" s="15"/>
+      <c r="BB41" s="12"/>
+      <c r="BC41" s="13"/>
+      <c r="BD41" s="13"/>
+      <c r="BE41" s="15"/>
+      <c r="BF41" s="12"/>
+      <c r="BG41" s="13"/>
+      <c r="BH41" s="13"/>
+      <c r="BI41" s="15"/>
+      <c r="BJ41" s="12"/>
+      <c r="BK41" s="13"/>
+      <c r="BL41" s="13"/>
+      <c r="BM41" s="15"/>
+    </row>
+    <row r="42" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>44</v>
       </c>
@@ -3271,11 +3976,27 @@
       <c r="AT42" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="AU42" s="22"/>
-      <c r="AV42" s="22"/>
+      <c r="AU42" s="19"/>
+      <c r="AV42" s="19"/>
       <c r="AW42" s="10"/>
-    </row>
-    <row r="43" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX42" s="25"/>
+      <c r="AY42" s="25"/>
+      <c r="AZ42" s="25"/>
+      <c r="BA42" s="26"/>
+      <c r="BB42" s="25"/>
+      <c r="BC42" s="25"/>
+      <c r="BD42" s="25"/>
+      <c r="BE42" s="26"/>
+      <c r="BF42" s="25"/>
+      <c r="BG42" s="25"/>
+      <c r="BH42" s="25"/>
+      <c r="BI42" s="26"/>
+      <c r="BJ42" s="25"/>
+      <c r="BK42" s="25"/>
+      <c r="BL42" s="25"/>
+      <c r="BM42" s="26"/>
+    </row>
+    <row r="43" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>45</v>
       </c>
@@ -3330,11 +4051,27 @@
       <c r="AT43" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="AU43" s="22"/>
-      <c r="AV43" s="22"/>
+      <c r="AU43" s="19"/>
+      <c r="AV43" s="19"/>
       <c r="AW43" s="10"/>
-    </row>
-    <row r="44" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX43" s="25"/>
+      <c r="AY43" s="25"/>
+      <c r="AZ43" s="25"/>
+      <c r="BA43" s="26"/>
+      <c r="BB43" s="25"/>
+      <c r="BC43" s="25"/>
+      <c r="BD43" s="25"/>
+      <c r="BE43" s="26"/>
+      <c r="BF43" s="25"/>
+      <c r="BG43" s="25"/>
+      <c r="BH43" s="25"/>
+      <c r="BI43" s="26"/>
+      <c r="BJ43" s="25"/>
+      <c r="BK43" s="25"/>
+      <c r="BL43" s="25"/>
+      <c r="BM43" s="26"/>
+    </row>
+    <row r="44" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>46</v>
       </c>
@@ -3389,11 +4126,27 @@
       <c r="AT44" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="AU44" s="22"/>
-      <c r="AV44" s="22"/>
+      <c r="AU44" s="19"/>
+      <c r="AV44" s="19"/>
       <c r="AW44" s="10"/>
-    </row>
-    <row r="45" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX44" s="25"/>
+      <c r="AY44" s="25"/>
+      <c r="AZ44" s="25"/>
+      <c r="BA44" s="26"/>
+      <c r="BB44" s="25"/>
+      <c r="BC44" s="25"/>
+      <c r="BD44" s="25"/>
+      <c r="BE44" s="26"/>
+      <c r="BF44" s="25"/>
+      <c r="BG44" s="25"/>
+      <c r="BH44" s="25"/>
+      <c r="BI44" s="26"/>
+      <c r="BJ44" s="25"/>
+      <c r="BK44" s="25"/>
+      <c r="BL44" s="25"/>
+      <c r="BM44" s="26"/>
+    </row>
+    <row r="45" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>47</v>
       </c>
@@ -3445,14 +4198,30 @@
       <c r="AS45" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="AT45" s="22"/>
+      <c r="AT45" s="19"/>
       <c r="AU45" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="AV45" s="22"/>
+      <c r="AV45" s="19"/>
       <c r="AW45" s="10"/>
-    </row>
-    <row r="46" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX45" s="25"/>
+      <c r="AY45" s="25"/>
+      <c r="AZ45" s="25"/>
+      <c r="BA45" s="26"/>
+      <c r="BB45" s="25"/>
+      <c r="BC45" s="25"/>
+      <c r="BD45" s="25"/>
+      <c r="BE45" s="26"/>
+      <c r="BF45" s="25"/>
+      <c r="BG45" s="25"/>
+      <c r="BH45" s="25"/>
+      <c r="BI45" s="26"/>
+      <c r="BJ45" s="25"/>
+      <c r="BK45" s="25"/>
+      <c r="BL45" s="25"/>
+      <c r="BM45" s="26"/>
+    </row>
+    <row r="46" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>48</v>
       </c>
@@ -3504,14 +4273,30 @@
       <c r="AS46" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="AT46" s="22"/>
+      <c r="AT46" s="19"/>
       <c r="AU46" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="AV46" s="22"/>
+      <c r="AV46" s="19"/>
       <c r="AW46" s="10"/>
-    </row>
-    <row r="47" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX46" s="25"/>
+      <c r="AY46" s="25"/>
+      <c r="AZ46" s="25"/>
+      <c r="BA46" s="26"/>
+      <c r="BB46" s="25"/>
+      <c r="BC46" s="25"/>
+      <c r="BD46" s="25"/>
+      <c r="BE46" s="26"/>
+      <c r="BF46" s="25"/>
+      <c r="BG46" s="25"/>
+      <c r="BH46" s="25"/>
+      <c r="BI46" s="26"/>
+      <c r="BJ46" s="25"/>
+      <c r="BK46" s="25"/>
+      <c r="BL46" s="25"/>
+      <c r="BM46" s="26"/>
+    </row>
+    <row r="47" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>49</v>
       </c>
@@ -3563,14 +4348,30 @@
       <c r="AS47" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="AT47" s="22"/>
+      <c r="AT47" s="19"/>
       <c r="AU47" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="AV47" s="22"/>
+      <c r="AV47" s="19"/>
       <c r="AW47" s="10"/>
-    </row>
-    <row r="48" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX47" s="25"/>
+      <c r="AY47" s="25"/>
+      <c r="AZ47" s="25"/>
+      <c r="BA47" s="26"/>
+      <c r="BB47" s="25"/>
+      <c r="BC47" s="25"/>
+      <c r="BD47" s="25"/>
+      <c r="BE47" s="26"/>
+      <c r="BF47" s="25"/>
+      <c r="BG47" s="25"/>
+      <c r="BH47" s="25"/>
+      <c r="BI47" s="26"/>
+      <c r="BJ47" s="25"/>
+      <c r="BK47" s="25"/>
+      <c r="BL47" s="25"/>
+      <c r="BM47" s="26"/>
+    </row>
+    <row r="48" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>50</v>
       </c>
@@ -3622,14 +4423,30 @@
       <c r="AS48" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="AT48" s="22"/>
-      <c r="AU48" s="22"/>
+      <c r="AT48" s="19"/>
+      <c r="AU48" s="19"/>
       <c r="AV48" s="17" t="s">
         <v>66</v>
       </c>
       <c r="AW48" s="10"/>
-    </row>
-    <row r="49" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX48" s="25"/>
+      <c r="AY48" s="25"/>
+      <c r="AZ48" s="25"/>
+      <c r="BA48" s="26"/>
+      <c r="BB48" s="25"/>
+      <c r="BC48" s="25"/>
+      <c r="BD48" s="25"/>
+      <c r="BE48" s="26"/>
+      <c r="BF48" s="25"/>
+      <c r="BG48" s="25"/>
+      <c r="BH48" s="25"/>
+      <c r="BI48" s="26"/>
+      <c r="BJ48" s="25"/>
+      <c r="BK48" s="25"/>
+      <c r="BL48" s="25"/>
+      <c r="BM48" s="26"/>
+    </row>
+    <row r="49" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>51</v>
       </c>
@@ -3681,14 +4498,30 @@
       <c r="AS49" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="AT49" s="22"/>
-      <c r="AU49" s="22"/>
+      <c r="AT49" s="19"/>
+      <c r="AU49" s="19"/>
       <c r="AV49" s="17" t="s">
         <v>66</v>
       </c>
       <c r="AW49" s="10"/>
-    </row>
-    <row r="50" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX49" s="25"/>
+      <c r="AY49" s="25"/>
+      <c r="AZ49" s="25"/>
+      <c r="BA49" s="26"/>
+      <c r="BB49" s="25"/>
+      <c r="BC49" s="25"/>
+      <c r="BD49" s="25"/>
+      <c r="BE49" s="26"/>
+      <c r="BF49" s="25"/>
+      <c r="BG49" s="25"/>
+      <c r="BH49" s="25"/>
+      <c r="BI49" s="26"/>
+      <c r="BJ49" s="25"/>
+      <c r="BK49" s="25"/>
+      <c r="BL49" s="25"/>
+      <c r="BM49" s="26"/>
+    </row>
+    <row r="50" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>52</v>
       </c>
@@ -3740,14 +4573,30 @@
       <c r="AS50" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="AT50" s="22"/>
-      <c r="AU50" s="22"/>
+      <c r="AT50" s="19"/>
+      <c r="AU50" s="19"/>
       <c r="AV50" s="17" t="s">
         <v>66</v>
       </c>
       <c r="AW50" s="10"/>
-    </row>
-    <row r="51" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX50" s="25"/>
+      <c r="AY50" s="25"/>
+      <c r="AZ50" s="25"/>
+      <c r="BA50" s="26"/>
+      <c r="BB50" s="25"/>
+      <c r="BC50" s="25"/>
+      <c r="BD50" s="25"/>
+      <c r="BE50" s="26"/>
+      <c r="BF50" s="25"/>
+      <c r="BG50" s="25"/>
+      <c r="BH50" s="25"/>
+      <c r="BI50" s="26"/>
+      <c r="BJ50" s="25"/>
+      <c r="BK50" s="25"/>
+      <c r="BL50" s="25"/>
+      <c r="BM50" s="26"/>
+    </row>
+    <row r="51" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>53</v>
       </c>
@@ -3799,14 +4648,30 @@
       <c r="AS51" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="AT51" s="22"/>
-      <c r="AU51" s="22"/>
-      <c r="AV51" s="22"/>
-      <c r="AW51" s="17" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="52" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AT51" s="19"/>
+      <c r="AU51" s="19"/>
+      <c r="AV51" s="19"/>
+      <c r="AW51" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="AX51" s="25"/>
+      <c r="AY51" s="25"/>
+      <c r="AZ51" s="25"/>
+      <c r="BA51" s="25"/>
+      <c r="BB51" s="25"/>
+      <c r="BC51" s="25"/>
+      <c r="BD51" s="25"/>
+      <c r="BE51" s="25"/>
+      <c r="BF51" s="25"/>
+      <c r="BG51" s="25"/>
+      <c r="BH51" s="25"/>
+      <c r="BI51" s="25"/>
+      <c r="BJ51" s="25"/>
+      <c r="BK51" s="25"/>
+      <c r="BL51" s="25"/>
+      <c r="BM51" s="25"/>
+    </row>
+    <row r="52" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>54</v>
       </c>
@@ -3894,12 +4759,28 @@
       <c r="AS52" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="AT52" s="23"/>
-      <c r="AU52" s="24"/>
-      <c r="AV52" s="24"/>
-      <c r="AW52" s="22"/>
-    </row>
-    <row r="53" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AT52" s="11"/>
+      <c r="AU52" s="9"/>
+      <c r="AV52" s="9"/>
+      <c r="AW52" s="10"/>
+      <c r="AX52" s="25"/>
+      <c r="AY52" s="28"/>
+      <c r="AZ52" s="28"/>
+      <c r="BA52" s="25"/>
+      <c r="BB52" s="25"/>
+      <c r="BC52" s="28"/>
+      <c r="BD52" s="28"/>
+      <c r="BE52" s="25"/>
+      <c r="BF52" s="25"/>
+      <c r="BG52" s="28"/>
+      <c r="BH52" s="28"/>
+      <c r="BI52" s="25"/>
+      <c r="BJ52" s="25"/>
+      <c r="BK52" s="28"/>
+      <c r="BL52" s="28"/>
+      <c r="BM52" s="25"/>
+    </row>
+    <row r="53" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>55</v>
       </c>
@@ -3991,8 +4872,24 @@
       <c r="AU53" s="9"/>
       <c r="AV53" s="9"/>
       <c r="AW53" s="10"/>
-    </row>
-    <row r="54" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX53" s="27"/>
+      <c r="AY53" s="28"/>
+      <c r="AZ53" s="28"/>
+      <c r="BA53" s="26"/>
+      <c r="BB53" s="27"/>
+      <c r="BC53" s="28"/>
+      <c r="BD53" s="28"/>
+      <c r="BE53" s="26"/>
+      <c r="BF53" s="27"/>
+      <c r="BG53" s="28"/>
+      <c r="BH53" s="28"/>
+      <c r="BI53" s="26"/>
+      <c r="BJ53" s="27"/>
+      <c r="BK53" s="28"/>
+      <c r="BL53" s="28"/>
+      <c r="BM53" s="26"/>
+    </row>
+    <row r="54" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>65</v>
       </c>
@@ -4045,8 +4942,24 @@
       </c>
       <c r="AU54" s="9"/>
       <c r="AV54" s="9"/>
-    </row>
-    <row r="55" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX54" s="29"/>
+      <c r="AY54" s="28"/>
+      <c r="AZ54" s="28"/>
+      <c r="BA54" s="30"/>
+      <c r="BB54" s="29"/>
+      <c r="BC54" s="28"/>
+      <c r="BD54" s="28"/>
+      <c r="BE54" s="30"/>
+      <c r="BF54" s="29"/>
+      <c r="BG54" s="28"/>
+      <c r="BH54" s="28"/>
+      <c r="BI54" s="30"/>
+      <c r="BJ54" s="29"/>
+      <c r="BK54" s="28"/>
+      <c r="BL54" s="28"/>
+      <c r="BM54" s="30"/>
+    </row>
+    <row r="55" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>56</v>
       </c>
@@ -4106,8 +5019,24 @@
       <c r="AW55" s="18" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="56" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX55" s="29"/>
+      <c r="AY55" s="25"/>
+      <c r="AZ55" s="25"/>
+      <c r="BA55" s="31"/>
+      <c r="BB55" s="29"/>
+      <c r="BC55" s="25"/>
+      <c r="BD55" s="25"/>
+      <c r="BE55" s="31"/>
+      <c r="BF55" s="29"/>
+      <c r="BG55" s="25"/>
+      <c r="BH55" s="25"/>
+      <c r="BI55" s="31"/>
+      <c r="BJ55" s="29"/>
+      <c r="BK55" s="25"/>
+      <c r="BL55" s="25"/>
+      <c r="BM55" s="31"/>
+    </row>
+    <row r="56" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>57</v>
       </c>
@@ -4237,8 +5166,24 @@
       <c r="AU56" s="9"/>
       <c r="AV56" s="9"/>
       <c r="AW56" s="10"/>
-    </row>
-    <row r="57" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AX56" s="11"/>
+      <c r="AY56" s="9"/>
+      <c r="AZ56" s="9"/>
+      <c r="BA56" s="10"/>
+      <c r="BB56" s="11"/>
+      <c r="BC56" s="9"/>
+      <c r="BD56" s="9"/>
+      <c r="BE56" s="10"/>
+      <c r="BF56" s="11"/>
+      <c r="BG56" s="9"/>
+      <c r="BH56" s="9"/>
+      <c r="BI56" s="10"/>
+      <c r="BJ56" s="11"/>
+      <c r="BK56" s="9"/>
+      <c r="BL56" s="9"/>
+      <c r="BM56" s="10"/>
+    </row>
+    <row r="57" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>58</v>
       </c>
@@ -4289,12 +5234,62 @@
       <c r="AT57" s="11"/>
       <c r="AU57" s="9"/>
       <c r="AV57" s="9"/>
-      <c r="AW57" s="18" t="s">
+      <c r="AW57" s="31"/>
+      <c r="AX57" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="AY57" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="AZ57" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="BA57" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="BB57" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="BC57" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="BD57" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="BE57" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="BF57" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="BG57" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="BH57" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="BI57" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="BJ57" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="BK57" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="BL57" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="BM57" s="18" t="s">
         <v>66</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="16">
+    <mergeCell ref="AX1:BA1"/>
+    <mergeCell ref="BB1:BE1"/>
+    <mergeCell ref="BF1:BI1"/>
+    <mergeCell ref="BJ1:BM1"/>
     <mergeCell ref="AT1:AW1"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="F1:I1"/>

</xml_diff>